<commit_message>
fix(excel): generate 100% ECMA-376 compliant XLSX template, improve parser robustness with coordinate mapping, clean download buffers, and add direct CSV template button
</commit_message>
<xml_diff>
--- a/storage/Template_Import_Siswa_Navasena.xlsx
+++ b/storage/Template_Import_Siswa_Navasena.xlsx
@@ -1,6 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22000" windowHeight="12000"/>
+  </bookViews>
   <sheets>
     <sheet name="Data Siswa" sheetId="1" r:id="rId1"/>
   </sheets>
@@ -10,100 +13,100 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
-    <t>nis</t>
-  </si>
-  <si>
-    <t>nama_lengkap</t>
-  </si>
-  <si>
-    <t>kelas</t>
-  </si>
-  <si>
-    <t>jenis_kelamin</t>
-  </si>
-  <si>
-    <t>telepon</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>20261001</t>
-  </si>
-  <si>
-    <t>Ahmad Fauzi</t>
-  </si>
-  <si>
-    <t>XII RPL 1</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>081234567801</t>
-  </si>
-  <si>
-    <t>ahmad.fauzi@smkn1panyingkiran.sch.id</t>
-  </si>
-  <si>
-    <t>20261002</t>
-  </si>
-  <si>
-    <t>Siti Nurhaliza</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>081234567802</t>
-  </si>
-  <si>
-    <t>siti.nurhaliza@smkn1panyingkiran.sch.id</t>
-  </si>
-  <si>
-    <t>20261003</t>
-  </si>
-  <si>
-    <t>Dimas Anggara</t>
-  </si>
-  <si>
-    <t>XII TKJ 1</t>
-  </si>
-  <si>
-    <t>081234567803</t>
-  </si>
-  <si>
-    <t>dimas.anggara@smkn1panyingkiran.sch.id</t>
-  </si>
-  <si>
-    <t>20261004</t>
-  </si>
-  <si>
-    <t>Dewi Lestari</t>
-  </si>
-  <si>
-    <t>XII AKL 1</t>
-  </si>
-  <si>
-    <t>081234567804</t>
-  </si>
-  <si>
-    <t>dewi.lestari@smkn1panyingkiran.sch.id</t>
-  </si>
-  <si>
-    <t>20261005</t>
-  </si>
-  <si>
-    <t>Rizky Pratama</t>
-  </si>
-  <si>
-    <t>XII TBSM 1</t>
-  </si>
-  <si>
-    <t>081234567805</t>
-  </si>
-  <si>
-    <t>rizky.pratama@smkn1panyingkiran.sch.id</t>
+    <t xml:space="preserve">nis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nama_lengkap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kelas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jenis_kelamin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">telepon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20261001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ahmad Fauzi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XII RPL 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">081234567801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ahmad.fauzi@smkn1panyingkiran.sch.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20261002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siti Nurhaliza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">081234567802</t>
+  </si>
+  <si>
+    <t xml:space="preserve">siti.nurhaliza@smkn1panyingkiran.sch.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20261003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimas Anggara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XII TKJ 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">081234567803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dimas.anggara@smkn1panyingkiran.sch.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20261004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dewi Lestari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XII AKL 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">081234567804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dewi.lestari@smkn1panyingkiran.sch.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20261005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rizky Pratama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XII TBSM 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">081234567805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rizky.pratama@smkn1panyingkiran.sch.id</t>
   </si>
 </sst>
 </file>
@@ -114,14 +117,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF0F172A"/>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -135,6 +138,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0B101D"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,6 +148,7 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -158,6 +163,7 @@
       <bottom style="thin">
         <color rgb="FFCBD5E1"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -168,21 +174,28 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" t="s" s="1">
         <v>0</v>
       </c>
@@ -202,7 +215,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" t="s" s="2">
         <v>6</v>
       </c>
@@ -222,7 +235,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" t="s" s="2">
         <v>12</v>
       </c>
@@ -242,7 +255,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" t="s" s="2">
         <v>17</v>
       </c>
@@ -262,7 +275,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="20" customHeight="1">
       <c r="A5" t="s" s="2">
         <v>22</v>
       </c>
@@ -282,7 +295,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="20" customHeight="1">
       <c r="A6" t="s" s="2">
         <v>27</v>
       </c>
@@ -303,5 +316,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>